<commit_message>
fix: etiquetar datos de ejemplo y endurecer seguridad
</commit_message>
<xml_diff>
--- a/01_bigpen_etl_bsale_pos/Caso01_BigPEN_Pipeline_ETL_Bsale_POS.xlsx
+++ b/01_bigpen_etl_bsale_pos/Caso01_BigPEN_Pipeline_ETL_Bsale_POS.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_Validacion_SKU_y_WSP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_Planilla_Importacion_Bsale" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_Resumen_KPIs_Jefatura" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Lee_esto" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Validacion_SKU_y_WSP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Planilla_Importacion_Bsale" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Resumen_KPIs_Jefatura" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +63,37 @@
       <color rgb="00065F46"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004B5563"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F2937"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -94,8 +124,18 @@
         <bgColor rgb="00065F46"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -131,11 +171,25 @@
         <color rgb="00E5E7EB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00F59E0B"/>
+      </left>
+      <right style="thin">
+        <color rgb="00F59E0B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00F59E0B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F59E0B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +204,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,7 +585,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="104" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>DATOS DE EJEMPLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>CASO 01 · LIBRERÍAS BIGPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>PIPELINE ETL, AUDITORÍA DE SKU Y MIGRACIÓN A BSALE POS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Los registros, descripciones, stock, costos y precios de este archivo son ficticios. Se usan solo para mostrar la lógica del pipeline, las fórmulas y los controles.
+Los SKU pueden coincidir con códigos públicos de productos, pero no representan datos comerciales reales de la empresa ni de sus clientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1"/>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Este aviso también aparece en el portafolio web y en el README del caso.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A6:D10"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -542,7 +676,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -936,18 +1069,28 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Datos de ejemplo: registros, stock, costos y precios ficticios. Los SKU pueden coincidir con códigos públicos, pero no son datos comerciales reales.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:H15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -974,7 +1117,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -1227,18 +1369,28 @@
         <v/>
       </c>
     </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Datos de ejemplo: registros, stock, costos y precios ficticios. Los SKU pueden coincidir con códigos públicos, pero no son datos comerciales reales.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:H12"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1253,7 +1405,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1356,7 +1507,17 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Datos de ejemplo: registros, stock, costos y precios ficticios. Los SKU pueden coincidir con códigos públicos, pero no son datos comerciales reales.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:C10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>